<commit_message>
second computer or license
</commit_message>
<xml_diff>
--- a/license_registry.xlsx
+++ b/license_registry.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Volumes/Ritesh_D/License_Easygraph/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CBF6FAC0-F5A9-7443-9B74-371AD5D95049}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0D8754AC-60EF-F841-AE96-0E04FB1B63FC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="29400" windowHeight="16660" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -83,7 +83,7 @@
     <t xml:space="preserve"> ea:1d:99:cf:f1:7b</t>
   </si>
   <si>
-    <t>ba:1e:98:cz:f1:8n</t>
+    <t>14-13-33-5E-F9-6D</t>
   </si>
 </sst>
 </file>

</xml_diff>

<commit_message>
mac bhi change kiya hai
</commit_message>
<xml_diff>
--- a/license_registry.xlsx
+++ b/license_registry.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Volumes/Ritesh_D/License_Easygraph/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{22A80BD2-E253-F94A-A81C-E891A6B62ABC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BE4CDCBD-9179-DB41-8DD5-DE467EF86558}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="29400" windowHeight="16660" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -83,7 +83,7 @@
     <t xml:space="preserve"> ea:1d:99:cf:f1:7b</t>
   </si>
   <si>
-    <t>14-13-33-5E-F9-6D</t>
+    <t>14-13-33-5E-F9-6C</t>
   </si>
 </sst>
 </file>

</xml_diff>

<commit_message>
MAC ADDRESS CHANGE IS ALSO WORKING
</commit_message>
<xml_diff>
--- a/license_registry.xlsx
+++ b/license_registry.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Volumes/Ritesh_D/License_Easygraph/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{38E420FB-D649-1F4E-A4F6-2EE03F3334D8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ED928DFD-BE57-AA43-8ED1-A94155B5070D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="29400" windowHeight="16660" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -89,7 +89,7 @@
     <t>50-5B-C2-EE-1A-89</t>
   </si>
   <si>
-    <t>14-13-33-5E-F9-6E</t>
+    <t>14-13-33-5E-F9-6D</t>
   </si>
 </sst>
 </file>
@@ -322,11 +322,11 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="49" fontId="2" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="2" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -678,10 +678,10 @@
       </c>
     </row>
     <row r="4" spans="1:3" ht="22" customHeight="1">
-      <c r="A4" s="17" t="s">
+      <c r="A4" s="16" t="s">
         <v>20</v>
       </c>
-      <c r="B4" s="17" t="s">
+      <c r="B4" s="16" t="s">
         <v>21</v>
       </c>
       <c r="C4" s="15" t="s">
@@ -824,12 +824,12 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="32" customHeight="1">
-      <c r="A1" s="16" t="s">
+      <c r="A1" s="17" t="s">
         <v>4</v>
       </c>
-      <c r="B1" s="16"/>
-      <c r="C1" s="16"/>
-      <c r="D1" s="16"/>
+      <c r="B1" s="17"/>
+      <c r="C1" s="17"/>
+      <c r="D1" s="17"/>
     </row>
     <row r="3" spans="1:4" ht="32" customHeight="1">
       <c r="A3" s="9" t="s">

</xml_diff>